<commit_message>
admin dashboard, public home page, timetable publishing features added
</commit_message>
<xml_diff>
--- a/classroom.xlsx
+++ b/classroom.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,6 +613,36 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CS-Year2-Comp1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CS-Year2-Comp2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Arts</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added dynamic daily workload balancing and improved empty slot labeling
</commit_message>
<xml_diff>
--- a/classroom.xlsx
+++ b/classroom.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A90355-A134-4365-A6C5-D8E864BEFF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="24">
   <si>
     <t>Classroom ID</t>
   </si>
@@ -62,19 +61,20 @@
     <t>2</t>
   </si>
   <si>
-    <t>Art</t>
-  </si>
-  <si>
     <t>CS-Year1-Comp1</t>
   </si>
   <si>
-    <t>Maths 1</t>
+    <r>
+      <t>Mathematics</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3</t>
+    </r>
   </si>
   <si>
     <t>Sports</t>
-  </si>
-  <si>
-    <t>CS-Year1-Comp1</t>
   </si>
   <si>
     <t>Physics</t>
@@ -95,14 +95,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -428,9 +428,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="27.77734375" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
@@ -438,7 +438,7 @@
     <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -460,7 +460,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -471,7 +471,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -482,7 +482,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -493,7 +493,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -504,7 +504,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -515,7 +515,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -537,7 +537,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -548,7 +548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -559,7 +559,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -570,7 +570,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -581,7 +581,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -592,31 +592,31 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>17</v>
       </c>
-      <c r="C16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
@@ -625,9 +625,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
         <v>13</v>
@@ -636,56 +636,56 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
         <v>19</v>
-      </c>
-      <c r="B19" t="s">
-        <v>20</v>
       </c>
       <c r="C19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" t="s">
         <v>21</v>
       </c>
-      <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" t="s">
-        <v>23</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
         <v>17</v>
       </c>
-      <c r="C22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" t="s">
         <v>18</v>
@@ -694,9 +694,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>13</v>
@@ -705,34 +705,34 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27">
         <v>5</v>

</xml_diff>